<commit_message>
M02 Lab 1: add Student Info + Declaration sheet and Setup(API key) sheet; VBA reads key from Setup!C7; restyle (no vertical borders, light headers, highlighted input cells)
</commit_message>
<xml_diff>
--- a/labs/M02/M02_Lab1_ExcelGPT_Starter.xlsx
+++ b/labs/M02/M02_Lab1_ExcelGPT_Starter.xlsx
@@ -7,12 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviews" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classify" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ask Anything" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Student Info" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regression" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviews" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classify" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ask Anything" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,12 +34,21 @@
     <font>
       <b val="1"/>
       <color rgb="00001A70"/>
-      <sz val="14"/>
+      <sz val="15"/>
     </font>
     <font>
       <i val="1"/>
-      <color rgb="00555555"/>
+      <color rgb="005A6B85"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="001E293B"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -46,7 +56,7 @@
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="00333333"/>
+      <color rgb="00334155"/>
       <sz val="10"/>
     </font>
     <font>
@@ -56,7 +66,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="002563EB"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -69,16 +79,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000055D4"/>
+        <fgColor rgb="00FFF6D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEF3FF"/>
+        <fgColor rgb="00DCE9FF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -86,22 +96,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00E5C97B"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="002563EB"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00DCE3EE"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,155 +500,91 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="78" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Excel GPT  -  Test Workbook</t>
+          <t>Module 2, Lab 1: Excel GPT</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>DADS 5250: Generative AI in Practice</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
+          <t>Student Information and Declaration</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>HOW TO USE THIS FILE</t>
-        </is>
-      </c>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>1. Press Alt + F11 to open the VBA editor.</t>
-        </is>
-      </c>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>2. Choose Insert then Module, and paste the ExcelGPT.bas code.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>3. In the code, replace the API_KEY line with your own OpenAI key.</t>
-        </is>
-      </c>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>4. Come back to any tab below and press Ctrl+Alt+F9 to run the examples.</t>
-        </is>
-      </c>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Declaration of Completion</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>THE FUNCTIONS YOU ARE TESTING</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5">
-        <f>GPT(prompt)                     Ask the AI anything.</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5">
-        <f>GPT_ASK(question, range)        Ask a question about a range of data.</f>
-        <v/>
-      </c>
-    </row>
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>I certify that the work in this lab is my own. I completed the exercises myself, I did not share my API key, and I followed the course academic integrity policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="13">
-      <c r="A13" s="5">
-        <f>GPT_CALC(instruction, range)    Let the AI do the math, returns a number.</f>
-        <v/>
-      </c>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Signature (type your full name)</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>AskSelection  (macro)            Select cells, run it, ask in a pop up box.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>THE TABS</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Sales        tabular data     -&gt; GPT_ASK and GPT_CALC</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Regression   two columns      -&gt; trend, slope, prediction</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Reviews      long text        -&gt; summary and sentiment</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Classify     short text       -&gt; label each row</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Ask Anything general prompts  -&gt; GPT and translation</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Reminder: never save your real API key into a file you share.</t>
-        </is>
-      </c>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A9:D11"/>
+    <mergeCell ref="B8:D8"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -626,7 +595,102 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="64" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="54" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Setup: Load the Tools and Add Your API Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Do this once. It takes about two minutes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Your OpenAI API key</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>-&gt;</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>1. Press Alt + F11 to open the VBA editor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>2. Choose Insert then Module.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>3. Open ExcelGPT.bas, copy all of it, and paste it into the module.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>4. Close the editor and come back to this tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>5. Paste your OpenAI API key into the highlighted cell to the right.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>6. Go to any use-case tab and press Ctrl + Alt + F9 to run the examples.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Keep your key safe. Never share this file with your key still in it.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -644,493 +708,328 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>Product_Category</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>Units_Sold</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="10" t="inlineStr">
         <is>
           <t>Returns</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="11" t="n">
         <v>45200</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="11" t="n">
         <v>320</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="11" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Clothing</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="11" t="n">
         <v>38100</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="11" t="n">
         <v>540</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="11" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="11" t="n">
         <v>52400</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="11" t="n">
         <v>410</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="11" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="11" t="n">
         <v>31800</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="11" t="n">
         <v>210</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="11" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Clothing</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="11" t="n">
         <v>41500</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="11" t="n">
         <v>600</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="11" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="11" t="n">
         <v>58700</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="11" t="n">
         <v>470</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="11" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="11" t="n">
         <v>29400</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="11" t="n">
         <v>190</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="11" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Clothing</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="11" t="n">
         <v>43600</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="11" t="n">
         <v>580</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="11" t="n">
         <v>28</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" s="11" t="n">
         <v>61200</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="11" t="n">
         <v>500</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="11" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" s="11" t="n">
         <v>34700</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="11" t="n">
         <v>230</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="11" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Clothing</t>
         </is>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" s="11" t="n">
         <v>39800</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="11" t="n">
         <v>560</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="11" t="n">
         <v>26</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Dec</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" s="11" t="n">
         <v>55300</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="11" t="n">
         <v>440</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="11" t="n">
         <v>9</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>TRY THESE</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>These show #NAME? until you paste the VBA module and add your key. Then press Ctrl+Alt+F9 to recalc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>These show #NAME? until you load the VBA and add your key on the Setup tab, then press Ctrl+Alt+F9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>Total revenue (AI does the sum)</t>
         </is>
       </c>
-      <c r="C20" s="7">
+      <c r="C21" s="13">
         <f>GPT_CALC("total revenue", C4:C15)</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>Which category earns the most?</t>
         </is>
       </c>
-      <c r="C21" s="7">
+      <c r="C22" s="13">
         <f>GPT_ASK("Which product category earns the most and by how much?", A3:E15)</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>Average units for Electronics</t>
         </is>
       </c>
-      <c r="C22" s="7">
+      <c r="C23" s="13">
         <f>GPT_CALC("average units sold for Electronics only", A3:E15)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ad Spend vs Sales</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Ad_Spend</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>1000</v>
-      </c>
-      <c r="B4" t="n">
-        <v>8200</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>2000</v>
-      </c>
-      <c r="B5" t="n">
-        <v>11500</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>3000</v>
-      </c>
-      <c r="B6" t="n">
-        <v>15100</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>4000</v>
-      </c>
-      <c r="B7" t="n">
-        <v>17800</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>5000</v>
-      </c>
-      <c r="B8" t="n">
-        <v>22400</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>6000</v>
-      </c>
-      <c r="B9" t="n">
-        <v>25100</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>7000</v>
-      </c>
-      <c r="B10" t="n">
-        <v>29800</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>8000</v>
-      </c>
-      <c r="B11" t="n">
-        <v>31200</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>9000</v>
-      </c>
-      <c r="B12" t="n">
-        <v>36500</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>10000</v>
-      </c>
-      <c r="B13" t="n">
-        <v>39100</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>TRY THESE</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>These show #NAME? until you paste the VBA module and add your key. Then press Ctrl+Alt+F9 to recalc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Describe the relationship</t>
-        </is>
-      </c>
-      <c r="C18" s="7">
-        <f>GPT_ASK("Describe the relationship between ad spend and sales.", A3:B13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Approximate slope (sales per $1 ad spend)</t>
-        </is>
-      </c>
-      <c r="C19" s="7">
-        <f>GPT_CALC("the slope of sales versus ad spend, as sales gained per one dollar of ad spend", A3:B13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Predict sales at 9500 ad spend</t>
-        </is>
-      </c>
-      <c r="C20" s="7">
-        <f>GPT_ASK("Predict the sales if ad spend is 9500, and briefly explain.", A3:B13)</f>
         <v/>
       </c>
     </row>
@@ -1145,113 +1044,157 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Customer Reviews</t>
+          <t>Ad Spend vs Sales</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Ad_Spend</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Sales</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>The setup was quick but the battery drains way too fast.</t>
-        </is>
+      <c r="A4" s="11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>8200</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Absolutely love it, best purchase I made this year!</t>
-        </is>
+      <c r="A5" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>11500</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Customer service never responded to my emails. Frustrating.</t>
-        </is>
+      <c r="A6" s="11" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>15100</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Good value for the price, though the packaging was damaged.</t>
-        </is>
+      <c r="A7" s="11" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>17800</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Works as described. Nothing special but it does the job.</t>
-        </is>
+      <c r="A8" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>22400</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>The app keeps crashing on my phone, very disappointing.</t>
-        </is>
+      <c r="A9" s="11" t="n">
+        <v>6000</v>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>25100</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="n">
+        <v>7000</v>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>29800</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="11" t="n">
+        <v>8000</v>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>31200</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="n">
+        <v>9000</v>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>36500</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="n">
+        <v>10000</v>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>39100</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>TRY THESE</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>These show #NAME? until you paste the VBA module and add your key. Then press Ctrl+Alt+F9 to recalc.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Summarize the main themes</t>
-        </is>
-      </c>
-      <c r="C14" s="7">
-        <f>GPT_ASK("Summarize the main themes across all these reviews in 2 sentences.", A3:A9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Overall sentiment</t>
-        </is>
-      </c>
-      <c r="C15" s="7">
-        <f>GPT_ASK("What is the overall sentiment, and what is the most common complaint?", A3:A9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Five word summary of one review</t>
-        </is>
-      </c>
-      <c r="C16" s="7">
-        <f>GPT("Summarize this review in five words: " &amp; A4)</f>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>These show #NAME? until you load the VBA and add your key on the Setup tab, then press Ctrl+Alt+F9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Describe the relationship</t>
+        </is>
+      </c>
+      <c r="C19" s="13">
+        <f>GPT_ASK("Describe the relationship between ad spend and sales.", A3:B13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Approximate slope</t>
+        </is>
+      </c>
+      <c r="C20" s="13">
+        <f>GPT_CALC("the slope of sales versus ad spend, as sales gained per one dollar", A3:B13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Predict sales at 9500</t>
+        </is>
+      </c>
+      <c r="C21" s="13">
+        <f>GPT_ASK("Predict the sales if ad spend is 9500, and briefly explain.", A3:B13)</f>
         <v/>
       </c>
     </row>
@@ -1266,121 +1209,113 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="64" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Classify Each Message</t>
+          <t>Customer Reviews</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Message</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>AI Label (put a formula in this column)</t>
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Review</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Shipping was super fast, thank you!</t>
-        </is>
-      </c>
-      <c r="B4" s="7">
-        <f>GPT("Classify as Positive, Negative, or Neutral. Reply with one word only: " &amp; A4)</f>
-        <v/>
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>The setup was quick but the battery drains way too fast.</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Item arrived broken and unusable.</t>
-        </is>
-      </c>
-      <c r="B5" s="7">
-        <f>GPT("Classify as Positive, Negative, or Neutral. Reply with one word only: " &amp; A5)</f>
-        <v/>
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Absolutely love it, best purchase I made this year!</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>It's okay, not great, not terrible.</t>
-        </is>
-      </c>
-      <c r="B6" s="7">
-        <f>GPT("Classify as Positive, Negative, or Neutral. Reply with one word only: " &amp; A6)</f>
-        <v/>
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Customer service never responded to my emails. Frustrating.</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Best coffee maker I have ever owned!</t>
-        </is>
-      </c>
-      <c r="B7" s="7">
-        <f>GPT("Classify as Positive, Negative, or Neutral. Reply with one word only: " &amp; A7)</f>
-        <v/>
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Good value for the price, though the packaging was damaged.</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Waited three weeks and still nothing.</t>
-        </is>
-      </c>
-      <c r="B8" s="7">
-        <f>GPT("Classify as Positive, Negative, or Neutral. Reply with one word only: " &amp; A8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>HOW IT WORKS</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>These show #NAME? until you paste the VBA module and add your key. Then press Ctrl+Alt+F9 to recalc.</t>
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Works as described. Nothing special but it does the job.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>The app keeps crashing on my phone, very disappointing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>TRY THESE</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Column B already has a formula per row.</t>
-        </is>
-      </c>
-      <c r="C13" s="7">
-        <f>GPT("Classify ... Reply one word only: " &amp; A4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Try your own</t>
-        </is>
-      </c>
-      <c r="C14" s="7">
-        <f>GPT("Is this message urgent? Reply Yes or No: " &amp; A4)</f>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>These show #NAME? until you load the VBA and add your key on the Setup tab, then press Ctrl+Alt+F9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Summarize the main themes</t>
+        </is>
+      </c>
+      <c r="C15" s="13">
+        <f>GPT_ASK("Summarize the main themes across all these reviews in 2 sentences.", A3:A9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Overall sentiment</t>
+        </is>
+      </c>
+      <c r="C16" s="13">
+        <f>GPT_ASK("What is the overall sentiment and the most common complaint?", A3:A9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Five word summary</t>
+        </is>
+      </c>
+      <c r="C17" s="13">
+        <f>GPT("Summarize this review in five words: " &amp; A4)</f>
         <v/>
       </c>
     </row>
@@ -1395,50 +1330,179 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Classify Each Message</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Message</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>AI Label</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Shipping was super fast, thank you!</t>
+        </is>
+      </c>
+      <c r="B4" s="14">
+        <f>GPT("Classify as Positive, Negative, or Neutral. Reply with one word only: " &amp; A4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Item arrived broken and unusable.</t>
+        </is>
+      </c>
+      <c r="B5" s="14">
+        <f>GPT("Classify as Positive, Negative, or Neutral. Reply with one word only: " &amp; A5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>It's okay, not great, not terrible.</t>
+        </is>
+      </c>
+      <c r="B6" s="14">
+        <f>GPT("Classify as Positive, Negative, or Neutral. Reply with one word only: " &amp; A6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Best coffee maker I have ever owned!</t>
+        </is>
+      </c>
+      <c r="B7" s="14">
+        <f>GPT("Classify as Positive, Negative, or Neutral. Reply with one word only: " &amp; A7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Waited three weeks and still nothing.</t>
+        </is>
+      </c>
+      <c r="B8" s="14">
+        <f>GPT("Classify as Positive, Negative, or Neutral. Reply with one word only: " &amp; A8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>HOW IT WORKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>These show #NAME? until you load the VBA and add your key on the Setup tab, then press Ctrl+Alt+F9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Column B already has a formula per row.</t>
+        </is>
+      </c>
+      <c r="C14" s="13">
+        <f>GPT("Classify ... one word only: " &amp; A4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Try your own</t>
+        </is>
+      </c>
+      <c r="C15" s="13">
+        <f>GPT("Is this message urgent? Reply Yes or No: " &amp; A4)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
           <t>General Prompts</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Maria</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>David</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Priya</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>TRY THESE</t>
         </is>
@@ -1447,39 +1511,39 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>These show #NAME? until you paste the VBA module and add your key. Then press Ctrl+Alt+F9 to recalc.</t>
+          <t>These show #NAME? until you load the VBA and add your key on the Setup tab, then press Ctrl+Alt+F9.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Ask for KPIs</t>
         </is>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="13">
         <f>GPT("Give me 3 KPIs a retail sales manager should track.")</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Translate to Spanish</t>
         </is>
       </c>
-      <c r="C12" s="7">
+      <c r="C12" s="13">
         <f>GPT("Translate to Spanish: Thank you for your order.")</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Write a thank you line</t>
         </is>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="13">
         <f>GPT("Write a one line thank you email to a customer named " &amp; A4)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
M02 Lab 1: add optional Model cell on Setup tab (C8); VBA reads model via GetModel() so students can switch models without editing code
</commit_message>
<xml_diff>
--- a/labs/M02/M02_Lab1_ExcelGPT_Starter.xlsx
+++ b/labs/M02/M02_Lab1_ExcelGPT_Starter.xlsx
@@ -88,7 +88,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -111,11 +111,20 @@
         <color rgb="00DCE3EE"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="002563EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -135,6 +144,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -554,6 +564,8 @@
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
+      <c r="C8" s="15" t="n"/>
+      <c r="D8" s="15" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -630,6 +642,30 @@
       </c>
       <c r="C7" s="8" t="n"/>
     </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Model (optional, advanced)</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>-&gt;</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>gpt-4.1-mini</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Leave the model as is unless you know you want a different one. gpt-4.1-mini is fast and cheap.</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
M02 Lab 1: set body text to 11pt across all tabs (titles kept larger)
</commit_message>
<xml_diff>
--- a/labs/M02/M02_Lab1_ExcelGPT_Starter.xlsx
+++ b/labs/M02/M02_Lab1_ExcelGPT_Starter.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,6 +69,25 @@
       <color rgb="002563EB"/>
       <sz val="11"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="005A6B85"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="00334155"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="00001A70"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -88,7 +107,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -120,11 +139,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <bottom style="medium">
+        <color rgb="002563EB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -145,6 +170,17 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -527,14 +563,14 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Student Information and Declaration</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>First Name</t>
         </is>
@@ -542,7 +578,7 @@
       <c r="B4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Last Name</t>
         </is>
@@ -550,7 +586,7 @@
       <c r="B5" s="4" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Student ID</t>
         </is>
@@ -563,12 +599,12 @@
           <t>Declaration of Completion</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n"/>
+      <c r="B8" s="18" t="n"/>
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="15" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>I certify that the work in this lab is my own. I completed the exercises myself, I did not share my API key, and I followed the course academic integrity policy.</t>
         </is>
@@ -577,7 +613,7 @@
     <row r="10"/>
     <row r="11"/>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Signature (type your full name)</t>
         </is>
@@ -585,7 +621,7 @@
       <c r="B13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
@@ -623,93 +659,93 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Do this once. It takes about two minutes.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Your OpenAI API key</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>-&gt;</t>
         </is>
       </c>
-      <c r="C7" s="8" t="n"/>
+      <c r="C7" s="20" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Model (optional, advanced)</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>-&gt;</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>gpt-4.1-mini</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Leave the model as is unless you know you want a different one. gpt-4.1-mini is fast and cheap.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>1. Press Alt + F11 to open the VBA editor.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>2. Choose Insert then Module.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>3. Open ExcelGPT.bas, copy all of it, and paste it into the module.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>4. Close the editor and come back to this tab.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>5. Paste your OpenAI API key into the highlighted cell to the right.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>6. Go to any use-case tab and press Ctrl + Alt + F9 to run the examples.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>Keep your key safe. Never share this file with your key still in it.</t>
         </is>
@@ -771,254 +807,254 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="C4" s="11" t="n">
+      <c r="C4" s="22" t="n">
         <v>45200</v>
       </c>
-      <c r="D4" s="11" t="n">
+      <c r="D4" s="22" t="n">
         <v>320</v>
       </c>
-      <c r="E4" s="11" t="n">
+      <c r="E4" s="22" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Clothing</t>
         </is>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="22" t="n">
         <v>38100</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="22" t="n">
         <v>540</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="22" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C6" s="22" t="n">
         <v>52400</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="22" t="n">
         <v>410</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="22" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C7" s="22" t="n">
         <v>31800</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D7" s="22" t="n">
         <v>210</v>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="22" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Clothing</t>
         </is>
       </c>
-      <c r="C8" s="11" t="n">
+      <c r="C8" s="22" t="n">
         <v>41500</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="22" t="n">
         <v>600</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="22" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="C9" s="11" t="n">
+      <c r="C9" s="22" t="n">
         <v>58700</v>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="22" t="n">
         <v>470</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="22" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="22" t="n">
         <v>29400</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="22" t="n">
         <v>190</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="22" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>Clothing</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="22" t="n">
         <v>43600</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="22" t="n">
         <v>580</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="22" t="n">
         <v>28</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="22" t="n">
         <v>61200</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="22" t="n">
         <v>500</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="22" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="22" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="22" t="n">
         <v>34700</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="22" t="n">
         <v>230</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="22" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="22" t="inlineStr">
         <is>
           <t>Clothing</t>
         </is>
       </c>
-      <c r="C14" s="11" t="n">
+      <c r="C14" s="22" t="n">
         <v>39800</v>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="22" t="n">
         <v>560</v>
       </c>
-      <c r="E14" s="11" t="n">
+      <c r="E14" s="22" t="n">
         <v>26</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>Dec</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B15" s="22" t="inlineStr">
         <is>
           <t>Electronics</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C15" s="22" t="n">
         <v>55300</v>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D15" s="22" t="n">
         <v>440</v>
       </c>
-      <c r="E15" s="11" t="n">
+      <c r="E15" s="22" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1030,41 +1066,41 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>These show #NAME? until you load the VBA and add your key on the Setup tab, then press Ctrl+Alt+F9.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>Total revenue (AI does the sum)</t>
         </is>
       </c>
-      <c r="C21" s="13">
+      <c r="C21" s="23">
         <f>GPT_CALC("total revenue", C4:C15)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="A22" s="21" t="inlineStr">
         <is>
           <t>Which category earns the most?</t>
         </is>
       </c>
-      <c r="C22" s="13">
+      <c r="C22" s="23">
         <f>GPT_ASK("Which product category earns the most and by how much?", A3:E15)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>Average units for Electronics</t>
         </is>
       </c>
-      <c r="C23" s="13">
+      <c r="C23" s="23">
         <f>GPT_CALC("average units sold for Electronics only", A3:E15)</f>
         <v/>
       </c>
@@ -1108,82 +1144,82 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="n">
+      <c r="A4" s="22" t="n">
         <v>1000</v>
       </c>
-      <c r="B4" s="11" t="n">
+      <c r="B4" s="22" t="n">
         <v>8200</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="n">
+      <c r="A5" s="22" t="n">
         <v>2000</v>
       </c>
-      <c r="B5" s="11" t="n">
+      <c r="B5" s="22" t="n">
         <v>11500</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="n">
+      <c r="A6" s="22" t="n">
         <v>3000</v>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="22" t="n">
         <v>15100</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n">
+      <c r="A7" s="22" t="n">
         <v>4000</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="22" t="n">
         <v>17800</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="n">
+      <c r="A8" s="22" t="n">
         <v>5000</v>
       </c>
-      <c r="B8" s="11" t="n">
+      <c r="B8" s="22" t="n">
         <v>22400</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n">
+      <c r="A9" s="22" t="n">
         <v>6000</v>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="22" t="n">
         <v>25100</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="22" t="n">
         <v>7000</v>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="22" t="n">
         <v>29800</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n">
+      <c r="A11" s="22" t="n">
         <v>8000</v>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="22" t="n">
         <v>31200</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n">
+      <c r="A12" s="22" t="n">
         <v>9000</v>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="22" t="n">
         <v>36500</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n">
+      <c r="A13" s="22" t="n">
         <v>10000</v>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="22" t="n">
         <v>39100</v>
       </c>
     </row>
@@ -1195,41 +1231,41 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>These show #NAME? until you load the VBA and add your key on the Setup tab, then press Ctrl+Alt+F9.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>Describe the relationship</t>
         </is>
       </c>
-      <c r="C19" s="13">
+      <c r="C19" s="23">
         <f>GPT_ASK("Describe the relationship between ad spend and sales.", A3:B13)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="A20" s="21" t="inlineStr">
         <is>
           <t>Approximate slope</t>
         </is>
       </c>
-      <c r="C20" s="13">
+      <c r="C20" s="23">
         <f>GPT_CALC("the slope of sales versus ad spend, as sales gained per one dollar", A3:B13)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>Predict sales at 9500</t>
         </is>
       </c>
-      <c r="C21" s="13">
+      <c r="C21" s="23">
         <f>GPT_ASK("Predict the sales if ad spend is 9500, and briefly explain.", A3:B13)</f>
         <v/>
       </c>
@@ -1267,42 +1303,42 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>The setup was quick but the battery drains way too fast.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Absolutely love it, best purchase I made this year!</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>Customer service never responded to my emails. Frustrating.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>Good value for the price, though the packaging was damaged.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>Works as described. Nothing special but it does the job.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>The app keeps crashing on my phone, very disappointing.</t>
         </is>
@@ -1316,41 +1352,41 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>These show #NAME? until you load the VBA and add your key on the Setup tab, then press Ctrl+Alt+F9.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>Summarize the main themes</t>
         </is>
       </c>
-      <c r="C15" s="13">
+      <c r="C15" s="23">
         <f>GPT_ASK("Summarize the main themes across all these reviews in 2 sentences.", A3:A9)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>Overall sentiment</t>
         </is>
       </c>
-      <c r="C16" s="13">
+      <c r="C16" s="23">
         <f>GPT_ASK("What is the overall sentiment and the most common complaint?", A3:A9)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>Five word summary</t>
         </is>
       </c>
-      <c r="C17" s="13">
+      <c r="C17" s="23">
         <f>GPT("Summarize this review in five words: " &amp; A4)</f>
         <v/>
       </c>
@@ -1394,56 +1430,56 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Shipping was super fast, thank you!</t>
         </is>
       </c>
-      <c r="B4" s="14">
+      <c r="B4" s="24">
         <f>GPT("Classify as Positive, Negative, or Neutral. Reply with one word only: " &amp; A4)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Item arrived broken and unusable.</t>
         </is>
       </c>
-      <c r="B5" s="14">
+      <c r="B5" s="24">
         <f>GPT("Classify as Positive, Negative, or Neutral. Reply with one word only: " &amp; A5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>It's okay, not great, not terrible.</t>
         </is>
       </c>
-      <c r="B6" s="14">
+      <c r="B6" s="24">
         <f>GPT("Classify as Positive, Negative, or Neutral. Reply with one word only: " &amp; A6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>Best coffee maker I have ever owned!</t>
         </is>
       </c>
-      <c r="B7" s="14">
+      <c r="B7" s="24">
         <f>GPT("Classify as Positive, Negative, or Neutral. Reply with one word only: " &amp; A7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>Waited three weeks and still nothing.</t>
         </is>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="24">
         <f>GPT("Classify as Positive, Negative, or Neutral. Reply with one word only: " &amp; A8)</f>
         <v/>
       </c>
@@ -1456,30 +1492,30 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>These show #NAME? until you load the VBA and add your key on the Setup tab, then press Ctrl+Alt+F9.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>Column B already has a formula per row.</t>
         </is>
       </c>
-      <c r="C14" s="13">
+      <c r="C14" s="23">
         <f>GPT("Classify ... one word only: " &amp; A4)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>Try your own</t>
         </is>
       </c>
-      <c r="C15" s="13">
+      <c r="C15" s="23">
         <f>GPT("Is this message urgent? Reply Yes or No: " &amp; A4)</f>
         <v/>
       </c>
@@ -1517,21 +1553,21 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Maria</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>David</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>Priya</t>
         </is>
@@ -1545,41 +1581,41 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>These show #NAME? until you load the VBA and add your key on the Setup tab, then press Ctrl+Alt+F9.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Ask for KPIs</t>
         </is>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="23">
         <f>GPT("Give me 3 KPIs a retail sales manager should track.")</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>Translate to Spanish</t>
         </is>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="23">
         <f>GPT("Translate to Spanish: Thank you for your order.")</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>Write a thank you line</t>
         </is>
       </c>
-      <c r="C13" s="13">
+      <c r="C13" s="23">
         <f>GPT("Write a one line thank you email to a customer named " &amp; A4)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
M02 Lab 1: add cost warning (full recalc re-runs all AI cells) + freeze-to-values tip on Setup tab and in guide
</commit_message>
<xml_diff>
--- a/labs/M02/M02_Lab1_ExcelGPT_Starter.xlsx
+++ b/labs/M02/M02_Lab1_ExcelGPT_Starter.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -88,8 +88,13 @@
       <color rgb="00001A70"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0092400E"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -106,8 +111,13 @@
         <fgColor rgb="00DCE9FF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE8CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -145,11 +155,16 @@
         <color rgb="002563EB"/>
       </bottom>
     </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="00D97706"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -181,6 +196,11 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -643,7 +663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="64" customWidth="1" min="1" max="1"/>
@@ -751,7 +771,39 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="25" t="inlineStr">
+        <is>
+          <t>Cost note (read this)</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="27" t="inlineStr">
+        <is>
+          <t>Each function calls the AI every time its cell recalculates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="27" t="inlineStr">
+        <is>
+          <t>Pressing Ctrl+Alt+F9 re-runs every AI cell on the sheet at once, and charges you for all of them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>When you like an answer, copy the cell and use Paste Special then Values to freeze it. A frozen cell becomes plain text and never calls the AI again.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B22:C22"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>